<commit_message>
feat: Refactor data loader and dialogue generation for enhanced flexibility and support for arbitrary scenarios
- Simplified case info parsing in `data_loader.py` to handle generic fields and numeric suffixes.
- Updated `DialogueBuilder` to remove unnecessary condition metadata.
- Changed case loader from `XiaoyingCaseLoader` to `SplitCaseLoader` for better modularity.
- Enhanced placeholder filling in `utterance.py` to support dynamic field replacement.
- Added CI workflow for automated testing and demo data generation.
- Introduced MIT license and comprehensive README for project documentation.
- Implemented numeric comparison conditions for flexible evaluation of case fields.
- Developed extensive unit tests for data loading, condition parsing, and path generation.
</commit_message>
<xml_diff>
--- a/demo/data/话术模板.xlsx
+++ b/demo/data/话术模板.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="身份确认" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="积分告知" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="无意愿" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="流失风险" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="承诺到店" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="已到店" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="语音留言" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="链接促销话术" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="身份确认" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="积分告知" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="无意愿" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="流失风险" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="承诺到店" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="已到店" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="语音留言" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="链接促销话术" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,13 +24,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -41,7 +44,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -49,12 +52,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -424,42 +436,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>uid</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>parent(继承)</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>repeat(次数)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>conditions(条件)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>human(客户)</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>assistant(专员)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>flexible_stop(可选不继承)</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>是否再见</t>
         </is>
@@ -568,42 +580,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>uid</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>parent(继承)</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>repeat(次数)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>conditions(条件)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>human(客户)</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>assistant(专员)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>flexible_stop(可选不继承)</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>是否再见</t>
         </is>
@@ -657,7 +669,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>积分可兑换{门店名称}指定饮品，消费时每100积分抵扣{应还金额}元 / 积分能兑换饮品，消费时每100积分可抵{应还金额}元</t>
+          <t>积分可兑换{门店名称}指定饮品，单笔消费满{消费金额}元可用积分抵扣 / 积分能兑换饮品，单笔消费满{消费金额}元即可用积分抵扣</t>
         </is>
       </c>
       <c r="G3" t="n">
@@ -712,42 +724,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>uid</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>parent(继承)</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>repeat(次数)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>conditions(条件)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>human(客户)</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>assistant(专员)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>flexible_stop(可选不继承)</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>是否再见</t>
         </is>
@@ -856,42 +868,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>uid</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>parent(继承)</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>repeat(次数)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>conditions(条件)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>human(客户)</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>assistant(专员)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>flexible_stop(可选不继承)</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>是否再见</t>
         </is>
@@ -1000,42 +1012,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>uid</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>parent(继承)</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>repeat(次数)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>conditions(条件)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>human(客户)</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>assistant(专员)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>flexible_stop(可选不继承)</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>是否再见</t>
         </is>
@@ -1114,42 +1126,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>uid</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>parent(继承)</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>repeat(次数)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>conditions(条件)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>human(客户)</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>assistant(专员)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>flexible_stop(可选不继承)</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>是否再见</t>
         </is>
@@ -1198,42 +1210,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>uid</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>parent(继承)</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>repeat(次数)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>conditions(条件)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>human(客户)</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>assistant(专员)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>flexible_stop(可选不继承)</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>是否再见</t>
         </is>
@@ -1278,42 +1290,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>uid</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>parent(继承)</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>repeat(次数)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>conditions(条件)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>human(客户)</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>assistant(专员)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>flexible_stop(可选不继承)</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>是否再见</t>
         </is>
@@ -1333,7 +1345,7 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>顺便跟您说下，{门店名称}本周有会员日双倍积分活动，消费满{应还金额}元额外赠送{随机金额}积分 / 另外提醒您{客户姓名}，本周会员日消费有双倍积分，满{应还金额}元还送{随机金额}积分</t>
+          <t>顺便跟您说下，{门店名称}本周有会员日双倍积分活动，消费满{消费金额}元额外赠送{随机金额}积分 / 另外提醒您{客户姓名}，本周会员日消费有双倍积分，满{消费金额}元还送{随机金额}积分</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -1363,7 +1375,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>还有储值充{应还金额}送{随机金额}的活动，{会员等级}会员额外加赠一杯饮品 / 储值充{应还金额}送{随机金额}，{会员等级}会员还额外赠送一杯饮品哦</t>
+          <t>还有储值充{消费金额}送{随机金额}的活动，{会员等级}会员额外加赠一杯饮品 / 储值充{消费金额}送{随机金额}，{会员等级}会员还额外赠送一杯饮品哦</t>
         </is>
       </c>
       <c r="G3" t="n">

</xml_diff>

<commit_message>
feat: Enhance demo configuration and data files for milk tea member callback scenario
</commit_message>
<xml_diff>
--- a/demo/data/话术模板.xlsx
+++ b/demo/data/话术模板.xlsx
@@ -1,28 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="身份确认" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="身份核实" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="积分告知" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="权益介绍" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="活动推荐" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="无意愿" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="犹豫跟进" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="承诺到店" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="预约到店" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="流失风险" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="投诉处理" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="语音留言" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="已到店" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="明确拒绝" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="通话结束" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="链接促销话术" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="身份确认" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="身份核实" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="积分告知" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="权益介绍" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="活动推荐" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="无意愿" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="犹豫跟进" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="承诺到店" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="预约到店" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="流失风险" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="投诉处理" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="语音留言" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="已到店" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="明确拒绝" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="通话结束" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="链接促销话术" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -32,16 +32,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -52,7 +49,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -60,21 +57,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -444,42 +432,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>uid</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>parent(继承)</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>repeat(次数)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>conditions(条件)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>human(客户)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>assistant(专员)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>flexible_stop(可选不继承)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>是否再见</t>
         </is>
@@ -588,42 +576,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>uid</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>parent(继承)</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>repeat(次数)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>conditions(条件)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>human(客户)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>assistant(专员)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>flexible_stop(可选不继承)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>是否再见</t>
         </is>
@@ -702,42 +690,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>uid</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>parent(继承)</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>repeat(次数)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>conditions(条件)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>human(客户)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>assistant(专员)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>flexible_stop(可选不继承)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>是否再见</t>
         </is>
@@ -816,42 +804,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>uid</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>parent(继承)</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>repeat(次数)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>conditions(条件)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>human(客户)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>assistant(专员)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>flexible_stop(可选不继承)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>是否再见</t>
         </is>
@@ -896,42 +884,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>uid</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>parent(继承)</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>repeat(次数)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>conditions(条件)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>human(客户)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>assistant(专员)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>flexible_stop(可选不继承)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>是否再见</t>
         </is>
@@ -980,42 +968,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>uid</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>parent(继承)</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>repeat(次数)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>conditions(条件)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>human(客户)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>assistant(专员)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>flexible_stop(可选不继承)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>是否再见</t>
         </is>
@@ -1064,42 +1052,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>uid</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>parent(继承)</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>repeat(次数)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>conditions(条件)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>human(客户)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>assistant(专员)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>flexible_stop(可选不继承)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>是否再见</t>
         </is>
@@ -1148,42 +1136,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>uid</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>parent(继承)</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>repeat(次数)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>conditions(条件)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>human(客户)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>assistant(专员)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>flexible_stop(可选不继承)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>是否再见</t>
         </is>
@@ -1288,42 +1276,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>uid</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>parent(继承)</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>repeat(次数)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>conditions(条件)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>human(客户)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>assistant(专员)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>flexible_stop(可选不继承)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>是否再见</t>
         </is>
@@ -1402,42 +1390,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>uid</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>parent(继承)</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>repeat(次数)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>conditions(条件)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>human(客户)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>assistant(专员)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>flexible_stop(可选不继承)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>是否再见</t>
         </is>
@@ -1610,42 +1598,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>uid</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>parent(继承)</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>repeat(次数)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>conditions(条件)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>human(客户)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>assistant(专员)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>flexible_stop(可选不继承)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>是否再见</t>
         </is>
@@ -1756,42 +1744,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>uid</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>parent(继承)</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>repeat(次数)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>conditions(条件)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>human(客户)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>assistant(专员)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>flexible_stop(可选不继承)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>是否再见</t>
         </is>
@@ -1906,42 +1894,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>uid</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>parent(继承)</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>repeat(次数)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>conditions(条件)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>human(客户)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>assistant(专员)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>flexible_stop(可选不继承)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>是否再见</t>
         </is>
@@ -2020,42 +2008,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>uid</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>parent(继承)</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>repeat(次数)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>conditions(条件)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>human(客户)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>assistant(专员)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>flexible_stop(可选不继承)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>是否再见</t>
         </is>
@@ -2134,42 +2122,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>uid</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>parent(继承)</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>repeat(次数)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>conditions(条件)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>human(客户)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>assistant(专员)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>flexible_stop(可选不继承)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>是否再见</t>
         </is>
@@ -2248,42 +2236,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>uid</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>parent(继承)</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>repeat(次数)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>conditions(条件)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>human(客户)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>assistant(专员)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>flexible_stop(可选不继承)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>是否再见</t>
         </is>

</xml_diff>

<commit_message>
feat: Update dialogue prompts in demo data generation script for enhanced member callback scenarios
</commit_message>
<xml_diff>
--- a/demo/data/话术模板.xlsx
+++ b/demo/data/话术模板.xlsx
@@ -1,28 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="身份确认" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="身份核实" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="积分告知" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="权益介绍" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="活动推荐" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="无意愿" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="犹豫跟进" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="承诺到店" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="预约到店" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="流失风险" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="投诉处理" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="语音留言" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="已到店" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="明确拒绝" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="通话结束" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="链接促销话术" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="身份确认" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="身份核实" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="积分告知" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="权益介绍" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="活动推荐" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="无意愿" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="犹豫跟进" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="承诺到店" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="预约到店" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="流失风险" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="投诉处理" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="语音留言" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="已到店" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="明确拒绝" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="通话结束" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="链接促销话术" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -32,13 +32,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -49,7 +52,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -57,12 +60,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -432,42 +444,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>uid</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>parent(继承)</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>repeat(次数)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>conditions(条件)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>human(客户)</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>assistant(专员)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>flexible_stop(可选不继承)</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>是否再见</t>
         </is>
@@ -486,12 +498,12 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>喂你好 / 您好 / 喂？ / 哪位啊</t>
+          <t>喂你好 / 您好 / 喂？ / 哪位啊 / 你好，请问哪位 / 喂，谁呀 / 你好 / 喂，说话</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>您好，请问是{客户姓名}{客户性别}吗 / 您好，请问是{客户姓氏}本人吗 / 请问是{客户姓名}的手机号吗</t>
+          <t>您好，请问是{客户姓名}{客户性别}吗 / 您好，请问是{客户姓氏}本人吗 / 请问是{客户姓名}的手机号吗 / 您好，请问是{客户姓氏}的电话吗 / 您好，麻烦确认下是{客户姓名}{客户性别}本人吗 / 喂您好，请问是{客户姓名}吗</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -516,12 +528,12 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>是的我是 / 对，是我 / 我就是，你说</t>
+          <t>是的我是 / 对，是我 / 我就是，你说 / 嗯，我是 / 对，请问你哪位 / 是我，怎么了 / 嗯对，什么事</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>{客户姓名}您好，我是{门店名称}{专员工号}号专员，今天致电想跟您做个会员回访 / 您好{客户姓氏}，我是{门店名称}的客服，工号{专员工号}，今天来电做个会员关怀回访</t>
+          <t>{客户姓名}您好，我是{门店名称}{专员工号}号专员，今天致电想跟您做个会员回访 / 您好{客户姓氏}，我是{门店名称}的客服，工号{专员工号}，今天来电做个会员关怀回访 / {客户姓氏}您好，我是{门店名称}会员中心的{专员工号}，占用您两分钟做个回访 / 您好，我是{门店名称}的会员专员{专员工号}，今天给您来电是做个会员服务回访 / {客户姓名}{客户性别}您好，我是{门店名称}客服{专员工号}，想跟您简单聊两句会员权益的事</t>
         </is>
       </c>
       <c r="G3" t="n">
@@ -546,12 +558,12 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>哦好的你说 / 嗯，什么事 / 你说吧我听着</t>
+          <t>哦好的你说 / 嗯，什么事 / 你说吧我听着 / 行，你说 / 嗯嗯请讲 / 什么事呀 / 哦，你讲</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>是这样的，您是我们{门店名称}的{会员等级}会员，想先跟您确认下最近的消费体验 / 感谢您接听，您在{门店名称}的会员等级是{会员等级}，今天主要做个简单回访</t>
+          <t>是这样的，您是我们{门店名称}的{会员等级}会员，想先跟您确认下最近的消费体验 / 感谢您接听，您在{门店名称}的会员等级是{会员等级}，今天主要做个简单回访 / 您作为我们{门店名称}的{会员等级}会员，这次来电主要是回访下您最近的到店体验 / 您是我们{会员等级}会员，最近店里有些会员专属的变化想跟您同步一下 / 简单跟您说下，这次主要是针对{会员等级}会员做个关怀回访，耽误您一两分钟</t>
         </is>
       </c>
       <c r="G4" t="n">
@@ -576,42 +588,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>uid</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>parent(继承)</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>repeat(次数)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>conditions(条件)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>human(客户)</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>assistant(专员)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>flexible_stop(可选不继承)</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>是否再见</t>
         </is>
@@ -630,12 +642,12 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>你们奶茶越来越难喝了 / 上次体验很差不想去了 / 不想喝你们家了</t>
+          <t>你们奶茶越来越难喝了 / 上次体验很差不想去了 / 不想喝你们家了 / 上次买的都不好喝 / 感觉没以前好喝了 / 最近几次都挺失望的</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>非常抱歉给您带来不好的体验，我们已经改进配方，还推出了好几款新品 / 听到您这么说很抱歉，您方便说下具体哪方面不满意吗，我们一定改进 / 对不起让您失望了，您的意见我们会认真对待</t>
+          <t>非常抱歉给您带来不好的体验，我们已经改进配方，还推出了好几款新品 / 听到您这么说很抱歉，您方便说下具体哪方面不满意吗，我们一定改进 / 对不起让您失望了，您的意见我们会认真对待 / 非常抱歉给您带来不好的体验，您能具体说说是哪款饮品或哪次消费吗 / 实在抱歉，方便说说是哪次体验不满意吗，我们一定改进 / 抱歉让您失望了，能告诉我是哪次消费体验不好吗</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -660,12 +672,12 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>说了也没用 / 新品有什么 / 改没改进谁知道</t>
+          <t>说了也没用 / 新品有什么 / 改没改进谁知道 / 新品好喝吗 / 真改进了吗 / 说了你们也不改</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>您的意见对我们很重要，这次想邀请您免费试喝新品，再给我们一次机会 / 新品有芝芝莓莓和杨枝甘露，{会员等级}会员首杯半价 / 这次新品是我们重新研发的，您尝了不满意随时反馈</t>
+          <t>您的意见对我们很重要，这次想邀请您免费试喝新品，再给我们一次机会 / 新品有芝芝莓莓和杨枝甘露，{会员等级}会员首杯半价 / 这次新品是我们重新研发的，您尝了不满意随时反馈 / 理解您的心情，我们本月新上了两款低糖饮品，给老客户准备了免费试喝券 / 您的反馈我已经记录，同时送您一张新品试喝券，欢迎再来检验 / 我已经如实记录，另外送您一份小料券，希望您再给次机会</t>
         </is>
       </c>
       <c r="G3" t="n">
@@ -690,42 +702,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>uid</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>parent(继承)</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>repeat(次数)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>conditions(条件)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>human(客户)</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>assistant(专员)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>flexible_stop(可选不继承)</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>是否再见</t>
         </is>
@@ -744,12 +756,12 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>我要投诉 / 你们店员态度太差 / 上次的订单有问题</t>
+          <t>我要投诉 / 你们店员态度太差 / 上次的订单有问题 / 我要反映个问题 / 你们服务不行 / 上次消费让我很不满意</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>非常抱歉给您带来困扰，我马上为您记录并转交门店负责人 / 对不起{客户姓氏}，您的投诉我会加急处理，一定给您一个答复 / 实在抱歉，您慢慢说，我逐条记录</t>
+          <t>非常抱歉给您带来困扰，我马上为您记录并转交门店负责人 / 对不起{客户姓氏}，您的投诉我会加急处理，一定给您一个答复 / 实在抱歉，您慢慢说，我逐条记录 / 非常抱歉，您慢慢说，我这边详细记录 / 实在不好意思，您请讲，我一定如实记录并反馈 / 抱歉给您添麻烦了，您详细说下经过，我马上记录</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -774,12 +786,12 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>那你们怎么解决 / 我要赔偿 / 总要有个说法吧</t>
+          <t>那你们怎么解决 / 我要赔偿 / 总要有个说法吧 / 这事怎么处理 / 你们得给我个交代 / 你们打算怎么办</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>作为补偿，已为您账户发放优惠券和额外积分，您查收下 / 我们为您准备了免单券，48小时内到账，希望能弥补这次体验 / 门店负责人会在今天内主动联系您，补偿方案一并告知</t>
+          <t>作为补偿，已为您账户发放优惠券和额外积分，您查收下 / 我们为您准备了免单券，48小时内到账，希望能弥补这次体验 / 门店负责人会在今天内主动联系您，补偿方案一并告知 / 您反馈的问题24小时内会有专人回复处理，同时给您账户补一张优惠券表达歉意 / 我已加急上报门店经理，另外给您补了张{优惠券}，请您留意小程序 / 门店会在24小时内联系您处理，小小心意已发到您的账户</t>
         </is>
       </c>
       <c r="G3" t="n">
@@ -804,42 +816,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>uid</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>parent(继承)</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>repeat(次数)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>conditions(条件)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>human(客户)</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>assistant(专员)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>flexible_stop(可选不继承)</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>是否再见</t>
         </is>
@@ -859,7 +871,7 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>您好{客户姓名}，这里是{门店名称}客服，您有{积分余额}分积分即将到期，有空请回电{门店电话} / 您好，{门店名称}温馨提示您的积分{到期日期}到期，详情请回电{门店电话} / {客户姓氏}您好，会员积分即将清零，方便时请回电咨询</t>
+          <t>您好{客户姓名}，这里是{门店名称}客服，您有{积分余额}分积分即将到期，有空请回电{门店电话} / 您好，{门店名称}温馨提示您的积分{到期日期}到期，详情请回电{门店电话} / {客户姓氏}您好，会员积分即将清零，方便时请回电咨询 / 您好{客户姓氏}，{门店名称}会员回访，您账户有未使用的会员权益，详情请回电{门店电话} / {客户姓名}您好，这里是{门店名称}，您有张会员优惠券快过期了，有空请回电{门店电话} / 您好，{门店名称}客服留言，您的{会员等级}会员权益有更新，方便时回电{门店电话}了解</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -884,42 +896,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>uid</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>parent(继承)</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>repeat(次数)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>conditions(条件)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>human(客户)</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>assistant(专员)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>flexible_stop(可选不继承)</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>是否再见</t>
         </is>
@@ -938,12 +950,12 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>我已经到店了 / 刚在你们店消费完 / 我今天去过店里了</t>
+          <t>我已经到店了 / 刚在你们店消费完 / 我今天去过店里了 / 我刚从店里出来 / 我昨天去过了 / 我现在就在店里</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>感谢您的光临，积分兑换已为您办理，欢迎下次再来 / 太好了，已为您核销积分，期待您下次光临{门店名称} / 谢谢您的支持，这次的积分也已到账，欢迎常来</t>
+          <t>感谢您的光临，积分兑换已为您办理，欢迎下次再来 / 太好了，已为您核销积分，期待您下次光临{门店名称} / 谢谢您的支持，这次的积分也已到账，欢迎常来 / 感谢您的支持，本次消费积分已入账，欢迎常来 / 好的，已为您登记到店，会员权益正常生效，欢迎常来 / 感谢光临{门店名称}，本次积分已到账，期待下次再见</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -968,42 +980,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>uid</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>parent(继承)</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>repeat(次数)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>conditions(条件)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>human(客户)</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>assistant(专员)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>flexible_stop(可选不继承)</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>是否再见</t>
         </is>
@@ -1022,12 +1034,12 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>不用了以后别打了 / 别再联系我 / 说了不需要</t>
+          <t>不用了以后别打了 / 别再联系我 / 说了不需要 / 以后别打来了 / 不需要，别打了 / 别给我打电话了</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>好的非常抱歉打扰您了，祝您生活愉快，再见 / 明白了，我们不会再致电，抱歉打扰，再见 / 好的尊重您的决定，不再打扰，再见</t>
+          <t>好的非常抱歉打扰您了，祝您生活愉快，再见 / 明白了，我们不会再致电，抱歉打扰，再见 / 好的尊重您的决定，不再打扰，再见 / 好的，已为您登记免打扰，抱歉打扰，再见 / 明白，这就把您移出回访名单，祝您生活愉快</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -1052,42 +1064,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>uid</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>parent(继承)</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>repeat(次数)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>conditions(条件)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>human(客户)</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>assistant(专员)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>flexible_stop(可选不继承)</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>是否再见</t>
         </is>
@@ -1106,12 +1118,12 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>那就先这样 / 我先忙了挂了 / 行了知道了</t>
+          <t>那就先这样 / 我先忙了挂了 / 行了知道了 / 先这样吧拜拜 / 嗯，挂了哈 / 先这样，我这边有事</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>好的不打扰您了，再见 / 感谢您的接听，再见 / 好的，祝您生活顺心，再见</t>
+          <t>好的不打扰您了，再见 / 感谢您的接听，再见 / 好的，祝您生活顺心，再见 / 好的，那不耽误您时间了，再见 / 感谢您的时间，再见 / 好的您先忙，再见</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -1136,42 +1148,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>uid</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>parent(继承)</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>repeat(次数)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>conditions(条件)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>human(客户)</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>assistant(专员)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>flexible_stop(可选不继承)</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>是否再见</t>
         </is>
@@ -1191,7 +1203,7 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>顺便提醒您，{门店名称}本周会员日双倍积分，消费满{消费金额}元额外赠送{随机金额}积分 / 另外{客户姓氏}，本周会员日消费积分翻倍，满{消费金额}元再送{随机金额}积分</t>
+          <t>顺便提醒您，{门店名称}本周会员日双倍积分，消费满{消费金额}元额外赠送{随机金额}积分 / 另外{客户姓氏}，本周会员日消费积分翻倍，满{消费金额}元再送{随机金额}积分 / 顺带一提，本周会员日到店消费双倍积分，满{消费金额}元还有加赠 / 另外跟您说下，会员日当天消费积分翻倍，满额再送{随机金额}积分 / 顺便说一句，这周到店消费满{消费金额}元，积分双倍还加赠{随机金额}分</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -1216,12 +1228,12 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>是吗，还有什么活动 / 还有别的优惠吗</t>
+          <t>是吗，还有什么活动 / 还有别的优惠吗 / 哦？说来听听 / 还有啥活动 / 嗯，继续说</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>还有储值充{消费金额}送{随机金额}的活动，{会员等级}会员加赠一杯饮品 / 储值活动也很划算，充{消费金额}元送{随机金额}元，会员还多送一杯 / 现在办储值卡，{会员等级}会员首充立减再加赠饮品</t>
+          <t>还有储值充{消费金额}送{随机金额}的活动，{会员等级}会员加赠一杯饮品 / 储值活动也很划算，充{消费金额}元送{随机金额}元，会员还多送一杯 / 现在办储值卡，{会员等级}会员首充立减再加赠饮品 / 另外储值满{消费金额}元送{随机金额}元，会员额外加赠招牌饮品 / 还有储值优惠，充{消费金额}送{随机金额}，{会员等级}会员再享折上折</t>
         </is>
       </c>
       <c r="G3" t="n">
@@ -1246,12 +1258,12 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>好的我看看 / 行，有空我去 / 知道了</t>
+          <t>好的我看看 / 行，有空我去 / 知道了 / 嗯，回头瞧瞧 / 好，我了解下</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>好的，活动详情可到{小程序名称}查看，到店咨询店员也行 / 活动详情小程序里都有，您到店直接问店员也可以 / 没问题，我把活动链接发您小程序消息</t>
+          <t>好的，活动详情可到{小程序名称}查看，到店咨询店员也行 / 活动详情小程序里都有，您到店直接问店员也可以 / 没问题，我把活动链接发您小程序消息 / 好的，您在{小程序名称}首页就能看到活动入口 / 行，活动详情我同步到您小程序消息里了</t>
         </is>
       </c>
       <c r="G4" t="n">
@@ -1276,42 +1288,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>uid</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>parent(继承)</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>repeat(次数)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>conditions(条件)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>human(客户)</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>assistant(专员)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>flexible_stop(可选不继承)</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>是否再见</t>
         </is>
@@ -1330,12 +1342,12 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>你怎么知道我电话的 / 你们从哪拿到的号码 / 谁让你们打电话的</t>
+          <t>你怎么知道我电话的 / 你们从哪拿到的号码 / 谁让你们打电话的 / 你们怎么会有我手机号 / 这号码你们哪来的 / 我没留过电话吧 / 你们是不是搞推销的</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>您别误会，是您在{小程序名称}注册会员时预留的号码，仅用于会员回访 / 您是我们{门店名称}的注册会员，信息只用于会员服务，请您放心</t>
+          <t>您别误会，是您在{小程序名称}注册会员时预留的号码，仅用于会员回访 / 您是我们{门店名称}的注册会员，信息只用于会员服务，请您放心 / 这个号码是您之前在{门店名称}办会员时登记的，仅做会员关怀使用 / 您放心，号码来自您在{小程序名称}的会员注册信息，不会用于其他用途 / 是您在门店消费注册会员时留的联系方式，我们只做回访，不做推销</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -1360,12 +1372,12 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>哦那行吧 / 好吧你说 / 行吧，长话短说</t>
+          <t>哦那行吧 / 好吧你说 / 行吧，长话短说 / 那你说吧 / 哦哦，那你讲 / 行，那你快说</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>好的谢谢理解，我这边简单跟您说下会员权益，耽误不了两分钟 / 感谢理解，那我就直说了</t>
+          <t>好的谢谢理解，我这边简单跟您说下会员权益，耽误不了两分钟 / 感谢理解，那我就直说了 / 谢谢您的信任，我长话短说 / 好的，简单说下您会员账户的最新情况 / 感谢您的理解，我尽快讲完不耽误您时间</t>
         </is>
       </c>
       <c r="G3" t="n">
@@ -1390,42 +1402,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>uid</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>parent(继承)</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>repeat(次数)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>conditions(条件)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>human(客户)</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>assistant(专员)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>flexible_stop(可选不继承)</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>是否再见</t>
         </is>
@@ -1444,12 +1456,12 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>积分还有多少 / 我的积分什么情况 / 我有多少积分来着</t>
+          <t>积分还有多少 / 我的积分什么情况 / 我有多少积分来着 / 帮我查下积分呗 / 积分还剩多少啊 / 我账户里还有多少分</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>您目前的积分余额是{积分余额}分 / 查到您账户里有{积分余额}积分 / 给您查了下，当前{积分余额}分</t>
+          <t>您目前的积分余额是{积分余额}分 / 查到您账户里有{积分余额}积分 / 给您查了下，当前{积分余额}分 / 您账户现在的积分余额是{积分余额}分 / 这边显示您还有{积分余额}分积分</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -1476,12 +1488,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>我积分这么多吗 / 这么多分啊 / 这么多积分能换不少吧</t>
+          <t>我积分这么多吗 / 这么多分啊 / 这么多积分能换不少吧 / 哇，有这么多呢 / 还真不少啊 / 我都不知道有这么多分</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>您的积分余额有{积分余额}分之多，属于我们的高积分会员 / 恭喜您{客户姓氏}，您有{积分余额}分积分，数额非常可观 / 您这积分量排在门店前百分之十呢</t>
+          <t>您的积分余额有{积分余额}分之多，属于我们的高积分会员 / 恭喜您{客户姓氏}，您有{积分余额}分积分，数额非常可观 / 您这积分量排在门店前百分之十呢 / 您是我们门店积分排名很靠前的会员了 / 您的积分积累得相当不错，{积分余额}分能换不少好东西</t>
         </is>
       </c>
       <c r="G3" t="n">
@@ -1508,12 +1520,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>才这么点 / 积分这么少啊 / 几乎没多少嘛</t>
+          <t>才这么点 / 积分这么少啊 / 几乎没多少嘛 / 就这么点分啊 / 哎，没多少积分 / 才几百分啊</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>您目前有{积分余额}分积分，额度不多，刚好可以趁活动攒一波 / 您的积分余额{积分余额}分，近期来消费顺便就能累积起来 / 分不多，配合活动用掉正合适</t>
+          <t>您目前有{积分余额}分积分，额度不多，刚好可以趁活动攒一波 / 您的积分余额{积分余额}分，近期来消费顺便就能累积起来 / 分不多，配合活动用掉正合适 / 现在{积分余额}分虽然不多，但最近活动多，很快就能攒起来 / 积分还不多，不过最近双倍积分活动挺适合您的</t>
         </is>
       </c>
       <c r="G4" t="n">
@@ -1538,12 +1550,12 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>那能怎么用 / 积分能干嘛 / 这积分有啥用</t>
+          <t>那能怎么用 / 积分能干嘛 / 这积分有啥用 / 积分可以换什么 / 这分能抵钱吗 / 积分怎么花划算</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>积分可以兑换{门店名称}的指定饮品，单笔消费满{消费金额}元就能用积分抵扣 / 积分既能换饮品也能抵现金，{会员等级}会员还有专属兑换价 / 每100积分抵1元，也能直接换招牌饮品</t>
+          <t>积分可以兑换{门店名称}的指定饮品，单笔消费满{消费金额}元就能用积分抵扣 / 积分既能换饮品也能抵现金，{会员等级}会员还有专属兑换价 / 每100积分抵1元，也能直接换招牌饮品 / 积分可以在小程序商城换饮品券，也能到店直接抵现 / 您的积分能兑换饮品，也能在会员日当现金抵扣用</t>
         </is>
       </c>
       <c r="G5" t="n">
@@ -1568,12 +1580,12 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>哦这样啊 / 我知道了 / 行吧</t>
+          <t>哦这样啊 / 我知道了 / 行吧 / 嗯，了解了 / 好的知道了 / 明白明白</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>温馨提示，您的积分在{到期日期}前有效，到期会清零，建议近期到店使用 / 提醒您一下，积分{到期日期}就到期了，抽空来用掉哦 / 别让积分白白过期，最近来一趟最划算</t>
+          <t>温馨提示，您的积分在{到期日期}前有效，到期会清零，建议近期到店使用 / 提醒您一下，积分{到期日期}就到期了，抽空来用掉哦 / 别让积分白白过期，最近来一趟最划算 / 您留意下，积分到{到期日期}就失效了，建议尽早安排 / 积分{到期日期}到期，早点来兑换别让分数浪费</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -1598,42 +1610,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>uid</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>parent(继承)</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>repeat(次数)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>conditions(条件)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>human(客户)</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>assistant(专员)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>flexible_stop(可选不继承)</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>是否再见</t>
         </is>
@@ -1652,12 +1664,12 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>会员有啥权益 / 你们会员有什么好处 / 会员能干啥</t>
+          <t>会员有啥权益 / 你们会员有什么好处 / 会员能干啥 / 会员有什么福利 / 入了会员有啥用 / 会员待遇怎么样</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>{会员等级}会员可享积分兑换、消费抵扣和生日礼遇 / 成为{门店名称}的{会员等级}会员，有积分抵现、专属折扣和新品试喝 / 权益主要是积分抵现、会员日折扣，还有每月一张优惠券</t>
+          <t>{会员等级}会员可享积分兑换、消费抵扣和生日礼遇 / 成为{门店名称}的{会员等级}会员，有积分抵现、专属折扣和新品试喝 / 权益主要是积分抵现、会员日折扣，还有每月一张优惠券 / {会员等级}会员能享受积分抵现、生日赠饮和会员日双倍积分 / 会员权益包括积分换饮品、专属优惠价，还有不定期的会员活动</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -1684,12 +1696,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>我这等级还有什么特别的 / 高等级有啥不一样</t>
+          <t>我这等级还有什么特别的 / 高等级有啥不一样 / 等级高有啥额外福利吗 / 会员等级高有啥好处 / 高等级会员能多享受什么</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>像您这样积分过千的{会员等级}会员，还能参加积分竞拍和限量周边兑换 / {会员等级}会员积分兑换打九折，每季还有一次免费升杯 / 高积分会员有专属客服通道和限定活动名额</t>
+          <t>像您这样积分过千的{会员等级}会员，还能参加积分竞拍和限量周边兑换 / {会员等级}会员积分兑换打九折，每季还有一次免费升杯 / 高积分会员有专属客服通道和限定活动名额 / 您这个等级还能享受新品优先试喝和生日双倍积分 / 积分高的会员每季度可以参与专属品鉴会</t>
         </is>
       </c>
       <c r="G3" t="n">
@@ -1714,12 +1726,12 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>还有呢 / 具体点 / 就这些啊</t>
+          <t>还有呢 / 具体点 / 就这些啊 / 还有别的吗 / 能再具体说说吗 / 别的福利呢</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>每周二是会员日，到店消费双倍积分，还能免费加一份小料 / 会员日当天{会员等级}会员第二杯半价，积分当钱花 / 生日当天来店里，饮品直接买一送一</t>
+          <t>每周二是会员日，到店消费双倍积分，还能免费加一份小料 / 会员日当天{会员等级}会员第二杯半价，积分当钱花 / 生日当天来店里，饮品直接买一送一 / 每月会员日消费满额还送限定周边 / 会员在小程序签到还能额外领积分</t>
         </is>
       </c>
       <c r="G4" t="n">
@@ -1744,42 +1756,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>uid</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>parent(继承)</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>repeat(次数)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>conditions(条件)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>human(客户)</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>assistant(专员)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>flexible_stop(可选不继承)</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>是否再见</t>
         </is>
@@ -1802,12 +1814,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>有什么活动吗 / 最近有优惠吗 / 这两天有啥活动</t>
+          <t>有什么活动吗 / 最近有优惠吗 / 这两天有啥活动 / 有啥优惠活动不 / 最近店里有什么活动 / 现在有什么优惠</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>看您账户里有张{优惠券}还没用，本周到店消费就能用 / 您有一张{优惠券}快过期了，趁这次活动用掉最划算 / 您账户的{优惠券}正好能和会员日叠加</t>
+          <t>看您账户里有张{优惠券}还没用，本周到店消费就能用 / 您有一张{优惠券}快过期了，趁这次活动用掉最划算 / 您账户的{优惠券}正好能和会员日叠加 / 您手里那张{优惠券}这周用正合适，还能叠加双倍积分 / 查到您有张{优惠券}没核销，本周活动叠加更划算</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -1834,12 +1846,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>没券就没活动了吗 / 不发券啊 / 还有别的吗</t>
+          <t>没券就没活动了吗 / 不发券啊 / 还有别的吗 / 没有券也有活动吧 / 别的活动呢 / 没券能参加什么</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>本周会员日双倍积分，消费满{消费金额}元还送{随机金额}积分 / 现在有新品半价活动，{会员等级}会员到店还能再减 / 没券也没关系，会员日当天积分翻倍一样划算</t>
+          <t>本周会员日双倍积分，消费满{消费金额}元还送{随机金额}积分 / 现在有新品半价活动，{会员等级}会员到店还能再减 / 没券也没关系，会员日当天积分翻倍一样划算 / 会员日当天全场第二杯半价，不限券 / 现在到店任意消费都能抽免单，会员中奖率更高</t>
         </is>
       </c>
       <c r="G3" t="n">
@@ -1864,12 +1876,12 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>是吗 / 那挺划算 / 哦？还有这种活动</t>
+          <t>是吗 / 那挺划算 / 哦？还有这种活动 / 听着不错 / 嗯，还行 / 真挺好 / 可以可以</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>活动到{到期日期}截止，您可以在{小程序名称}里先领券 / 名额有限，您在小程序下单还能额外获赠积分 / 活动详情我发您小程序消息里了，点开就能看</t>
+          <t>活动到{到期日期}截止，您可以在{小程序名称}里先领券 / 名额有限，您在小程序下单还能额外获赠积分 / 活动详情我发您小程序消息里了，点开就能看 / 活动就到{到期日期}，建议您提前在小程序预约 / 这个活动挺抢手的，您可以在{小程序名称}先看看详情</t>
         </is>
       </c>
       <c r="G4" t="n">
@@ -1894,42 +1906,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>uid</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>parent(继承)</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>repeat(次数)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>conditions(条件)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>human(客户)</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>assistant(专员)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>flexible_stop(可选不继承)</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>是否再见</t>
         </is>
@@ -1948,12 +1960,12 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>我不怎么去你们店了 / 算了不用了 / 暂时不需要</t>
+          <t>我不怎么去你们店了 / 算了不用了 / 暂时不需要 / 最近不太想买奶茶 / 不用了谢谢 / 最近不怎么喝奶茶了</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>理解您{客户姓氏}，不过您{积分余额}分积分不用就浪费了，要不要考虑来一趟 / 没关系，就是特意提醒您积分{到期日期}到期，别浪费了 / 好的不强求，顺带提醒下您的积分情况</t>
+          <t>理解您{客户姓氏}，不过您{积分余额}分积分不用就浪费了，要不要考虑来一趟 / 没关系，就是特意提醒您积分{到期日期}到期，别浪费了 / 好的不强求，顺带提醒下您的积分情况 / 理解理解，主要是您的积分快到期了，提醒您一下 / 没关系的{客户姓氏}，只是您的会员权益快到期了，觉得可惜才提醒您</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -1978,12 +1990,12 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>最近没时间 / 改天再说吧 / 以后吧 / 忙着呢</t>
+          <t>最近没时间 / 改天再说吧 / 以后吧 / 忙着呢 / 这阵子忙 / 过阵子再说 / 最近没空去</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>好的不打扰您，活动长期有效，您随时可以来{门店名称} / 没问题，您有空在{小程序名称}点单也能参与，不用专门跑一趟 / 行，那我加您个小程序消息，您有空了看</t>
+          <t>好的不打扰您，活动长期有效，您随时可以来{门店名称} / 没问题，您有空在{小程序名称}点单也能参与，不用专门跑一趟 / 行，那我加您个小程序消息，您有空了看 / 好的，您忙完在小程序下单也一样能用积分 / 那您先忙，权益信息我同步到您小程序账户里了</t>
         </is>
       </c>
       <c r="G3" t="n">
@@ -2008,42 +2020,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>uid</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>parent(继承)</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>repeat(次数)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>conditions(条件)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>human(客户)</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>assistant(专员)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>flexible_stop(可选不继承)</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>是否再见</t>
         </is>
@@ -2062,12 +2074,12 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>我再想想 / 让我考虑一下 / 再说吧 / 回头看情况</t>
+          <t>我再想想 / 让我考虑一下 / 再说吧 / 回头看情况 / 我考虑考虑 / 嗯……先不着急 / 想好了再说</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>没问题，您主要顾虑哪方面呢，我帮您介绍下 / 可以的，您是担心没时间还是优惠力度，我给您详细说说 / 理解，货比三家很正常，您想了解什么我都说清楚</t>
+          <t>没问题，您主要顾虑哪方面呢，我帮您介绍下 / 可以的，您是担心没时间还是优惠力度，我给您详细说说 / 理解，货比三家很正常，您想了解什么我都说清楚 / 好的不着急，您是对活动还是积分使用有疑问 / 您慢慢考虑，有什么不清楚的我现在就能解答</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -2092,12 +2104,12 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>也没啥顾虑就是懒 / 主要是太远了 / 最近天热不想出门</t>
+          <t>也没啥顾虑就是懒 / 主要是太远了 / 最近天热不想出门 / 懒得跑一趟 / 下雨天不想动 / 门店离我有点远</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>理解，您也可以在{小程序名称}点外卖，积分一样能用 / 那您忙的时候小程序下单，门店直接给您配送到家 / 不用专门跑，外卖下单会员权益照样享受</t>
+          <t>理解，您也可以在{小程序名称}点外卖，积分一样能用 / 那您忙的时候小程序下单，门店直接给您配送到家 / 不用专门跑，外卖下单会员权益照样享受 / 小程序下单满{消费金额}元免配送费，积分照样累积 / 您线上下单选择就近门店配送，权益和到店一样</t>
         </is>
       </c>
       <c r="G3" t="n">
@@ -2122,42 +2134,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>uid</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>parent(继承)</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>repeat(次数)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>conditions(条件)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>human(客户)</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>assistant(专员)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>flexible_stop(可选不继承)</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>是否再见</t>
         </is>
@@ -2176,12 +2188,12 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>行那我这两天去 / 好的我去看看 / 那我抽空去一趟</t>
+          <t>行那我这两天去 / 好的我去看看 / 那我抽空去一趟 / 可以，周末我去 / 行，这几天就去 / 好，明天顺路去</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>好的{客户姓氏}，期待您到店，有问题可拨打{门店电话} / 太好了，活动详情已发到您{小程序名称}账户，到店出示会员码就行 / 好嘞，您来之前可以小程序先点单，到店直接取</t>
+          <t>好的{客户姓氏}，期待您到店，有问题可拨打{门店电话} / 太好了，活动详情已发到您{小程序名称}账户，到店出示会员码就行 / 好嘞，您来之前可以小程序先点单，到店直接取 / 太好了，到店报手机号就能使用优惠，期待您的光临 / 好的，到店出示会员码即可，门店在商场负一层扶梯旁 / 欢迎光临，到店找店员核销就行</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -2206,12 +2218,12 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>好的谢谢 / 行那就这样 / 嗯，没问题</t>
+          <t>好的谢谢 / 行那就这样 / 嗯，没问题 / 好，谢啦 / 好的再见 / 嗯嗯，拜拜</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>感谢您的接听，祝您生活愉快，再见 / 谢谢您，再见，{门店名称}随时欢迎您 / 好的，祝您今天愉快，再见</t>
+          <t>感谢您的接听，祝您生活愉快，再见 / 谢谢您，再见，{门店名称}随时欢迎您 / 好的，祝您今天愉快，再见 / 不客气，祝您生活愉快，再见 / 好的，有问题随时联系门店，再见 / 好，期待您到店，再见</t>
         </is>
       </c>
       <c r="G3" t="n">
@@ -2236,42 +2248,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>uid</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>parent(继承)</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>repeat(次数)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>conditions(条件)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>human(客户)</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>assistant(专员)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>flexible_stop(可选不继承)</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>是否再见</t>
         </is>
@@ -2290,12 +2302,12 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>能预约吗 / 帮我留个名额 / 周末去人多不多</t>
+          <t>能预约吗 / 帮我留个名额 / 周末去人多不多 / 可以提前预约吗 / 能帮我订个位置吗 / 周末去要排队吗</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>可以的，您在{小程序名称}选好门店和时间预约就行，到店免排队 / 我帮您登记，预约到店出示会员码即可核销 / 周末位置紧张，提前预约我们给您留好</t>
+          <t>可以的，您在{小程序名称}选好门店和时间预约就行，到店免排队 / 我帮您登记，预约到店出示会员码即可核销 / 周末位置紧张，提前预约我们给您留好 / 当然可以，会员预约免排队，您定个时间 / 可以的，告诉我大概几点，我帮您登记 / 没问题，您说个时间我马上帮您约上</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -2320,12 +2332,12 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>好的那我约周末 / 行约好了 / 帮我约周六下午吧</t>
+          <t>好的那我约周末 / 行约好了 / 帮我约周六下午吧 / 那就约明天下午 / 约周日中午吧 / 帮我约周五晚上</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>已为您备注周末到店，期待您的光临，再见 / 好的，门店会提前为您准备，再见 / 登记好了，我们周六见，祝您生活愉快</t>
+          <t>已为您备注周末到店，期待您的光临，再见 / 好的，门店会提前为您准备，再见 / 登记好了，我们周六见，祝您生活愉快 / 已帮您预约成功，到店出示小程序预约码即可，期待光临 / 预约完成，{门店名称}随时恭候您 / 好的约好了，到店直接报手机号</t>
         </is>
       </c>
       <c r="G3" t="n">

</xml_diff>